<commit_message>
Fix bug with parseTask output
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -437,10 +437,10 @@
         <v>Requirements</v>
       </c>
       <c r="C2" s="1" t="d">
-        <v>2024-01-06T00:00:00.000Z</v>
+        <v>2024-01-05T17:00:00.000Z</v>
       </c>
       <c r="D2" s="1" t="d">
-        <v>2024-01-08T00:00:00.000Z</v>
+        <v>2024-01-07T17:00:00.000Z</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -457,10 +457,10 @@
         <v>Mockups</v>
       </c>
       <c r="C3" s="1" t="d">
-        <v>2024-01-09T00:00:00.000Z</v>
+        <v>2024-01-08T17:00:00.000Z</v>
       </c>
       <c r="D3" s="1" t="d">
-        <v>2024-01-12T00:00:00.000Z</v>
+        <v>2024-01-11T17:00:00.000Z</v>
       </c>
       <c r="E3">
         <v>3</v>
@@ -477,10 +477,10 @@
         <v>Review mockups</v>
       </c>
       <c r="C4" s="1" t="d">
-        <v>2024-01-12T00:00:00.000Z</v>
+        <v>2024-01-11T17:00:00.000Z</v>
       </c>
       <c r="D4" s="1" t="d">
-        <v>2024-01-17T00:00:00.000Z</v>
+        <v>2024-01-16T17:00:00.000Z</v>
       </c>
       <c r="E4">
         <v>5</v>
@@ -497,10 +497,10 @@
         <v>Backend</v>
       </c>
       <c r="C5" s="1" t="d">
-        <v>2024-01-15T00:00:00.000Z</v>
+        <v>2024-01-14T17:00:00.000Z</v>
       </c>
       <c r="D5" s="1" t="d">
-        <v>2024-01-27T00:00:00.000Z</v>
+        <v>2024-01-26T17:00:00.000Z</v>
       </c>
       <c r="E5">
         <v>12</v>
@@ -517,10 +517,10 @@
         <v>Frontend</v>
       </c>
       <c r="C6" s="1" t="d">
-        <v>2024-01-27T00:00:00.000Z</v>
+        <v>2024-01-26T17:00:00.000Z</v>
       </c>
       <c r="D6" s="1" t="d">
-        <v>2024-02-06T00:00:00.000Z</v>
+        <v>2024-02-05T17:00:00.000Z</v>
       </c>
       <c r="E6">
         <v>10</v>
@@ -537,10 +537,10 @@
         <v>Launch</v>
       </c>
       <c r="C7" s="1" t="d">
-        <v>2024-02-06T00:00:00.000Z</v>
+        <v>2024-02-05T17:00:00.000Z</v>
       </c>
       <c r="D7" s="1" t="d">
-        <v>2024-02-06T00:00:00.000Z</v>
+        <v>2024-02-05T17:00:00.000Z</v>
       </c>
       <c r="E7">
         <v>0</v>

</xml_diff>

<commit_message>
Swap main excel library to get visual bars
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -1,59 +1,225 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="A Sample Project" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="A Sample Project" state="visible" r:id="rId4"/>
   </sheets>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="47">
+  <si>
+    <t>A Sample Project</t>
+  </si>
+  <si>
+    <t>Section</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>Days</t>
+  </si>
+  <si>
+    <t>01-06</t>
+  </si>
+  <si>
+    <t>01-07</t>
+  </si>
+  <si>
+    <t>01-08</t>
+  </si>
+  <si>
+    <t>01-09</t>
+  </si>
+  <si>
+    <t>01-10</t>
+  </si>
+  <si>
+    <t>01-11</t>
+  </si>
+  <si>
+    <t>01-12</t>
+  </si>
+  <si>
+    <t>01-13</t>
+  </si>
+  <si>
+    <t>01-14</t>
+  </si>
+  <si>
+    <t>01-15</t>
+  </si>
+  <si>
+    <t>01-16</t>
+  </si>
+  <si>
+    <t>01-17</t>
+  </si>
+  <si>
+    <t>01-18</t>
+  </si>
+  <si>
+    <t>01-19</t>
+  </si>
+  <si>
+    <t>01-20</t>
+  </si>
+  <si>
+    <t>01-21</t>
+  </si>
+  <si>
+    <t>01-22</t>
+  </si>
+  <si>
+    <t>01-23</t>
+  </si>
+  <si>
+    <t>01-24</t>
+  </si>
+  <si>
+    <t>01-25</t>
+  </si>
+  <si>
+    <t>01-26</t>
+  </si>
+  <si>
+    <t>01-27</t>
+  </si>
+  <si>
+    <t>01-28</t>
+  </si>
+  <si>
+    <t>01-29</t>
+  </si>
+  <si>
+    <t>01-30</t>
+  </si>
+  <si>
+    <t>01-31</t>
+  </si>
+  <si>
+    <t>02-01</t>
+  </si>
+  <si>
+    <t>02-02</t>
+  </si>
+  <si>
+    <t>02-03</t>
+  </si>
+  <si>
+    <t>02-04</t>
+  </si>
+  <si>
+    <t>02-05</t>
+  </si>
+  <si>
+    <t>02-06</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>Requirements</t>
+  </si>
+  <si>
+    <t>Mockups</t>
+  </si>
+  <si>
+    <t>Review mockups</t>
+  </si>
+  <si>
+    <t>Build</t>
+  </si>
+  <si>
+    <t>Backend</t>
+  </si>
+  <si>
+    <t>Frontend</t>
+  </si>
+  <si>
+    <t>Launch</t>
+  </si>
+  <si>
+    <t>◆</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="60" formatCode="yyyy-mm-dd"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFECEFF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF43A047"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E88E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF26A69A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE53935"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFB8C00"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -61,19 +227,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFB0BEC5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -398,160 +595,313 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AK8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="36.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
+    <col min="3" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="37" width="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Section</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Task</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Start Date</v>
-      </c>
-      <c r="D1" t="str">
-        <v>End Date</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Duration (days)</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Tags</v>
-      </c>
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
+      <c r="AD1" s="1"/>
+      <c r="AE1" s="1"/>
+      <c r="AF1" s="1"/>
+      <c r="AG1" s="1"/>
+      <c r="AH1" s="1"/>
+      <c r="AI1" s="1"/>
+      <c r="AJ1" s="1"/>
+      <c r="AK1" s="1"/>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Design</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Requirements</v>
-      </c>
-      <c r="C2" s="1" t="d">
-        <v>2024-01-05T17:00:00.000Z</v>
-      </c>
-      <c r="D2" s="1" t="d">
-        <v>2024-01-07T17:00:00.000Z</v>
-      </c>
-      <c r="E2">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" t="str">
-        <v>done</v>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z2" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AC2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AD2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="AE2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="AF2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AG2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="AH2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="AI2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="AJ2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK2" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Design</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Mockups</v>
-      </c>
-      <c r="C3" s="1" t="d">
-        <v>2024-01-08T17:00:00.000Z</v>
-      </c>
-      <c r="D3" s="1" t="d">
-        <v>2024-01-11T17:00:00.000Z</v>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="4">
+        <v>45297</v>
+      </c>
+      <c r="D3" s="4">
+        <v>45299</v>
       </c>
       <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="4">
+        <v>45300</v>
+      </c>
+      <c r="D4" s="4">
+        <v>45303</v>
+      </c>
+      <c r="E4">
         <v>3</v>
       </c>
-      <c r="F3" t="str">
-        <v>active</v>
-      </c>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Design</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Review mockups</v>
-      </c>
-      <c r="C4" s="1" t="d">
-        <v>2024-01-11T17:00:00.000Z</v>
-      </c>
-      <c r="D4" s="1" t="d">
-        <v>2024-01-16T17:00:00.000Z</v>
-      </c>
-      <c r="E4">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="4">
+        <v>45303</v>
+      </c>
+      <c r="D5" s="4">
+        <v>45308</v>
+      </c>
+      <c r="E5">
         <v>5</v>
       </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Build</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Backend</v>
-      </c>
-      <c r="C5" s="1" t="d">
-        <v>2024-01-14T17:00:00.000Z</v>
-      </c>
-      <c r="D5" s="1" t="d">
-        <v>2024-01-26T17:00:00.000Z</v>
-      </c>
-      <c r="E5">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="4">
+        <v>45306</v>
+      </c>
+      <c r="D6" s="4">
+        <v>45318</v>
+      </c>
+      <c r="E6">
         <v>12</v>
       </c>
-      <c r="F5" t="str">
-        <v>crit</v>
-      </c>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="8"/>
+      <c r="S6" s="8"/>
+      <c r="T6" s="8"/>
+      <c r="U6" s="8"/>
+      <c r="V6" s="8"/>
+      <c r="W6" s="8"/>
+      <c r="X6" s="8"/>
+      <c r="Y6" s="8"/>
+      <c r="Z6" s="8"/>
     </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Build</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Frontend</v>
-      </c>
-      <c r="C6" s="1" t="d">
-        <v>2024-01-26T17:00:00.000Z</v>
-      </c>
-      <c r="D6" s="1" t="d">
-        <v>2024-02-05T17:00:00.000Z</v>
-      </c>
-      <c r="E6">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="4">
+        <v>45318</v>
+      </c>
+      <c r="D7" s="4">
+        <v>45328</v>
+      </c>
+      <c r="E7">
         <v>10</v>
       </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
+      <c r="AA7" s="7"/>
+      <c r="AB7" s="7"/>
+      <c r="AC7" s="7"/>
+      <c r="AD7" s="7"/>
+      <c r="AE7" s="7"/>
+      <c r="AF7" s="7"/>
+      <c r="AG7" s="7"/>
+      <c r="AH7" s="7"/>
+      <c r="AI7" s="7"/>
+      <c r="AJ7" s="7"/>
     </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Build</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Launch</v>
-      </c>
-      <c r="C7" s="1" t="d">
-        <v>2024-02-05T17:00:00.000Z</v>
-      </c>
-      <c r="D7" s="1" t="d">
-        <v>2024-02-05T17:00:00.000Z</v>
-      </c>
-      <c r="E7">
+    <row r="8" spans="1:37" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="4">
+        <v>45328</v>
+      </c>
+      <c r="D8" s="4">
+        <v>45328</v>
+      </c>
+      <c r="E8">
         <v>0</v>
       </c>
-      <c r="F7" t="str">
-        <v>milestone</v>
+      <c r="AK8" s="9" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
-  </ignoredErrors>
+  <mergeCells count="1">
+    <mergeCell ref="A1:AK1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>